<commit_message>
Convert four appendix tables to figures; add concept-MLP to cross-method values
Supervisor feedback: too many tables. Render the appendix concept-coverage,
sample-stability, register-convergence and cross-method value tables as
figures (fig10-fig13) generated by plot_figures.py from the same frozen
pipeline artifacts (fail-closed cross-checks against the published values),
and swap them into dissertation.tex (appendix now 5 figures / 15 tables,
main text untouched). Extend h1_cross_method_gap_values.py (v3) with
concept-retrieval LR + MLP columns (MLP spans axes per scope decisions;
zero-shot stays MPNet-only). Renumber the final bundle (Table29-33 retire,
Fig08-11 added), update collect_final_outputs.py, the word-helper census
(31 tables / 58 separator rows / 17 debris cells) and the build_word.sh
resource path. Rebuild dissertation.pdf/.docx.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/4_outputs/final/Table06.xlsx
+++ b/4_outputs/final/Table06.xlsx
@@ -417,13 +417,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,399 +439,909 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Keyword %</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Concept %</t>
+          <t>Semantic gaps</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Coverage predictors</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr"/>
+      <c r="H1" s="1" t="inlineStr"/>
+      <c r="I1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+0.3</t>
+          <t>Adj.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Reg.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cov.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SDom</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Res %</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pol %</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>No Poverty</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>0.827</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.6</t>
+          <t>0.440</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+0.387</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>-3.9</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>25.7</t>
+          <t>Zero Hunger</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25.7</t>
+          <t>0.428</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.0</t>
+          <t>0.137</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+0.291</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>Good Health</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>0.663</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-7.3</t>
+          <t>0.454</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>+0.209</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>21.0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>+21.0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>25.7</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>0.402</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.2</t>
+          <t>0.224</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>+0.178</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>+3.5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.575</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.2</t>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>+0.241</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-3.3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>5.1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>Clean Water</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>0.384</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+0.6</t>
+          <t>0.180</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+0.204</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-2.9</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>3.7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>Clean Energy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>0.514</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+0.1</t>
+          <t>0.242</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+0.272</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>+0.4</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>Decent Work</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+5.8</t>
+          <t>0.363</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>+0.262</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-2.0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>Innovation</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.421</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>0.330</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>+0.092</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>21.6</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>+21.6</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>25.9</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>4.3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>Reduced Ineq.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>0.458</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+2.9</t>
+          <t>0.312</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>+0.146</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-2.1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2.9</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>Sust. Cities</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>0.693</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.458</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>+0.236</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>+1.2</t>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>+2.7</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5.3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>Consumption</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0.280</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>+0.120</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-0.9</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>3.5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>Climate</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.598</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-0.3</t>
+          <t>0.266</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>+0.332</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-7.1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>11.3</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>Life Below Water</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>0.504</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>0.253</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>+0.251</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3.8</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>Life on Land</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>0.346</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.4</t>
+          <t>0.139</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>+0.207</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-2.1</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>Peace &amp; Justice</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.541</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.0</t>
+          <t>0.327</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>+0.214</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-8.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>17.3</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Spearman ρ = 0.948; Kendall = 0.868</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Partnerships</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.312</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.521</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>-0.210</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-11.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0.511</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.309</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>+0.202</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>+0.0</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>